<commit_message>
Corrected formating for all json files. Corrected contant for 1965 and 1966
</commit_message>
<xml_diff>
--- a/Notes/progress.xlsx
+++ b/Notes/progress.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t xml:space="preserve">Year</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t xml:space="preserve">done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Key_26</t>
   </si>
 </sst>
 </file>
@@ -182,19 +179,22 @@
       <c r="A3" s="2" t="n">
         <v>1965</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
         <f aca="false">A3+1</f>
         <v>1966</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
@@ -203,12 +203,8 @@
         <f aca="false">A4+1</f>
         <v>1967</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
@@ -217,12 +213,8 @@
         <f aca="false">A5+1</f>
         <v>1968</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
@@ -231,12 +223,8 @@
         <f aca="false">A6+1</f>
         <v>1969</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
@@ -245,12 +233,8 @@
         <f aca="false">A7+1</f>
         <v>1970</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
@@ -262,9 +246,7 @@
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
-      <c r="E9" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="E9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="n">

</xml_diff>